<commit_message>
Ghi quyết định: Khanh nhận TNF 東京企画 từ 11/2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GJjWaqKTGo1Zrw6K7RRJy3
</commit_message>
<xml_diff>
--- a/docs/tai-ve/Phan-tich-khoi-luong-MD-APIC.xlsx
+++ b/docs/tai-ve/Phan-tich-khoi-luong-MD-APIC.xlsx
@@ -79,7 +79,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">bàn giao cho Khanh (đề xuất 11/2026, muộn nhất 12/2026); điều phối xuất hàng chung cả nhóm; quản lý chung may mẫu</t>
+      <t xml:space="preserve">bàn giao cho Khanh từ 11/2026; điều phối xuất hàng chung cả nhóm; quản lý chung may mẫu</t>
     </r>
   </si>
   <si>
@@ -153,7 +153,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(nhận từ Cuong); hỗ trợ TNF </t>
+      <t xml:space="preserve">(nhận từ Cuong từ 11/2026); hỗ trợ TNF </t>
     </r>
     <r>
       <rPr>
@@ -482,7 +482,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">A. Chỉ các việc đã quyết (NW → Khanh ngay; TNF </t>
+      <t xml:space="preserve">A. Phương án cũ: NW → Khanh ngay; TNF </t>
     </r>
     <r>
       <rPr>
@@ -499,7 +499,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">và 1/3 mẫu TNF → Khanh từ 12/2026)</t>
+      <t xml:space="preserve">và 1/3 mẫu TNF → Khanh từ 12/2026</t>
     </r>
   </si>
   <si>
@@ -525,7 +525,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">C. B + chuyển TNF </t>
+      <t xml:space="preserve">C. B + TNF </t>
     </r>
     <r>
       <rPr>
@@ -533,7 +533,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">東京企画 </t>
+      <t xml:space="preserve">東京企画 → </t>
     </r>
     <r>
       <rPr>
@@ -542,7 +542,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">cho Khanh ngay từ 11/2026</t>
+      <t xml:space="preserve">Khanh từ 11/2026 (đã quyết 28/10/2026)</t>
     </r>
   </si>
   <si>
@@ -4682,7 +4682,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="36.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Loại 8 dòng cũ (Snowpeak, Montbell 23SS/23FW) bị đẩy ngày trong Plantable
Dòng 1976–1983 chuyền AP1B-9B: ô START dòng 1976 gõ cứng 28/11/2026, các
dòng sau nối tiếp bằng công thức nên đơn 2022–2023 hiện vào 11/2026–4/2027.
Tính lại tải theo tháng, cập nhật bản Word/Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GJjWaqKTGo1Zrw6K7RRJy3
</commit_message>
<xml_diff>
--- a/docs/tai-ve/Phan-tich-khoi-luong-MD-APIC.xlsx
+++ b/docs/tai-ve/Phan-tich-khoi-luong-MD-APIC.xlsx
@@ -324,10 +324,10 @@
     <t xml:space="preserve">Hien</t>
   </si>
   <si>
-    <t xml:space="preserve">Teton Bros, ALLTERRAIN, Mont-Bell, DESCENTE GOLF, Snowpeak (4 lô trên Plantable)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Không giao thêm. Tháng 11–12 khá cao (mẫu SKI, 14 mã vào chuyền tháng 12)</t>
+    <t xml:space="preserve">Teton Bros, ALLTERRAIN, Mont-Bell, DESCENTE GOLF, Snowpeak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Không giao thêm. Tháng 11–12 khá cao (mẫu SKI, 12 mã vào chuyền tháng 12)</t>
   </si>
   <si>
     <t xml:space="preserve">Nhu</t>
@@ -5483,25 +5483,25 @@
         <v>70</v>
       </c>
       <c r="C5" s="13" t="n">
-        <v>1.88</v>
+        <v>1.89</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>1.69</v>
+        <v>1.73</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>0.15</v>
       </c>
       <c r="F5" s="13" t="n">
-        <v>1.41</v>
+        <v>1.42</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>1.63</v>
+        <v>1.65</v>
       </c>
       <c r="H5" s="13" t="n">
-        <v>1.51</v>
+        <v>1.48</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5512,22 +5512,22 @@
         <v>71</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>2.16</v>
+        <v>2.21</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>1.9</v>
+        <v>1.94</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>1.61</v>
+        <v>1.5</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>0.35</v>
@@ -5541,25 +5541,25 @@
         <v>72</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>1.3</v>
+        <v>1.32</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>1.93</v>
+        <v>1.96</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>0.15</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>1.57</v>
+        <v>1.61</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>0.97</v>
+        <v>0.89</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>1.15</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5570,25 +5570,25 @@
         <v>73</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>1.29</v>
+        <v>1.31</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>0.11</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>0.47</v>
+        <v>0.48</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>0.68</v>
+        <v>0.54</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>0.79</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5599,25 +5599,25 @@
         <v>70</v>
       </c>
       <c r="C9" s="13" t="n">
-        <v>1.88</v>
+        <v>1.89</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>1.27</v>
+        <v>1.3</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>1.41</v>
+        <v>1.42</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>1.63</v>
+        <v>1.65</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>1.51</v>
+        <v>1.48</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5628,22 +5628,22 @@
         <v>71</v>
       </c>
       <c r="C10" s="13" t="n">
-        <v>2.16</v>
+        <v>2.21</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>1.43</v>
+        <v>1.46</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>1.23</v>
+        <v>1.25</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
       <c r="H10" s="13" t="n">
-        <v>1.61</v>
+        <v>1.5</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>0.35</v>
@@ -5657,25 +5657,25 @@
         <v>72</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>1.3</v>
+        <v>1.32</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>1.25</v>
+        <v>1.27</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>0.8</v>
+        <v>0.81</v>
       </c>
       <c r="F11" s="10" t="n">
         <v>0.15</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>1.57</v>
+        <v>1.61</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>0.97</v>
+        <v>0.89</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>1.15</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5686,25 +5686,25 @@
         <v>73</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>1.29</v>
+        <v>1.31</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="F12" s="10" t="n">
         <v>0.11</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.47</v>
+        <v>0.48</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>0.68</v>
+        <v>0.54</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>0.79</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5715,25 +5715,25 @@
         <v>70</v>
       </c>
       <c r="C13" s="13" t="n">
-        <v>1.69</v>
+        <v>1.71</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>1.27</v>
+        <v>1.3</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
       <c r="F13" s="13" t="n">
-        <v>1.41</v>
+        <v>1.42</v>
       </c>
       <c r="G13" s="13" t="n">
-        <v>1.63</v>
+        <v>1.65</v>
       </c>
       <c r="H13" s="13" t="n">
-        <v>1.51</v>
+        <v>1.48</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5744,22 +5744,22 @@
         <v>71</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>2.16</v>
+        <v>2.21</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>1.43</v>
+        <v>1.46</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>1.23</v>
+        <v>1.25</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
       <c r="H14" s="13" t="n">
-        <v>1.61</v>
+        <v>1.5</v>
       </c>
       <c r="I14" s="10" t="n">
         <v>0.35</v>
@@ -5773,25 +5773,25 @@
         <v>72</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>1.3</v>
+        <v>1.32</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>1.25</v>
+        <v>1.27</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>0.8</v>
+        <v>0.81</v>
       </c>
       <c r="F15" s="10" t="n">
         <v>0.15</v>
       </c>
       <c r="G15" s="13" t="n">
-        <v>1.57</v>
+        <v>1.61</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>0.97</v>
+        <v>0.89</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>1.15</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5802,25 +5802,25 @@
         <v>73</v>
       </c>
       <c r="C16" s="10" t="n">
-        <v>1.29</v>
+        <v>1.31</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="F16" s="10" t="n">
         <v>0.11</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>0.47</v>
+        <v>0.48</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>0.68</v>
+        <v>0.54</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>0.79</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5831,25 +5831,25 @@
         <v>70</v>
       </c>
       <c r="C17" s="13" t="n">
-        <v>1.69</v>
+        <v>1.71</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>1.27</v>
+        <v>1.3</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
       <c r="F17" s="13" t="n">
-        <v>1.41</v>
+        <v>1.42</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>1.63</v>
+        <v>1.65</v>
       </c>
       <c r="H17" s="13" t="n">
-        <v>1.51</v>
+        <v>1.48</v>
       </c>
       <c r="I17" s="10" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5860,22 +5860,22 @@
         <v>71</v>
       </c>
       <c r="C18" s="13" t="n">
-        <v>1.62</v>
+        <v>1.65</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>1.43</v>
+        <v>1.46</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>1.23</v>
+        <v>1.25</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>0.93</v>
+        <v>0.94</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>1.61</v>
+        <v>1.5</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>0.35</v>
@@ -5889,25 +5889,25 @@
         <v>72</v>
       </c>
       <c r="C19" s="10" t="n">
-        <v>1.3</v>
+        <v>1.32</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>1.25</v>
+        <v>1.27</v>
       </c>
       <c r="E19" s="10" t="n">
-        <v>0.8</v>
+        <v>0.81</v>
       </c>
       <c r="F19" s="10" t="n">
-        <v>0.47</v>
+        <v>0.48</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>1.26</v>
+        <v>1.29</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>0.97</v>
+        <v>0.89</v>
       </c>
       <c r="I19" s="10" t="n">
-        <v>1.15</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5918,25 +5918,25 @@
         <v>73</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>1.29</v>
+        <v>1.31</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="F20" s="10" t="n">
         <v>0.11</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.47</v>
+        <v>0.48</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>0.68</v>
+        <v>0.54</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>0.79</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5947,25 +5947,25 @@
         <v>70</v>
       </c>
       <c r="C21" s="13" t="n">
-        <v>1.69</v>
+        <v>1.71</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>1.27</v>
+        <v>1.3</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
       <c r="F21" s="13" t="n">
-        <v>1.41</v>
+        <v>1.42</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>1.63</v>
+        <v>1.65</v>
       </c>
       <c r="H21" s="13" t="n">
-        <v>1.51</v>
+        <v>1.48</v>
       </c>
       <c r="I21" s="10" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5975,26 +5975,26 @@
       <c r="B22" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="C22" s="10" t="n">
-        <v>1.38</v>
+      <c r="C22" s="13" t="n">
+        <v>1.41</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>1.43</v>
+        <v>1.46</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>1.23</v>
+        <v>1.25</v>
       </c>
       <c r="F22" s="10" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>0.93</v>
+        <v>0.94</v>
       </c>
       <c r="H22" s="13" t="n">
-        <v>1.61</v>
+        <v>1.5</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>0.56</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6005,25 +6005,25 @@
         <v>72</v>
       </c>
       <c r="C23" s="10" t="n">
-        <v>1.3</v>
+        <v>1.32</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>1.25</v>
+        <v>1.27</v>
       </c>
       <c r="E23" s="10" t="n">
-        <v>0.8</v>
+        <v>0.81</v>
       </c>
       <c r="F23" s="10" t="n">
-        <v>0.47</v>
+        <v>0.48</v>
       </c>
       <c r="G23" s="10" t="n">
-        <v>1.26</v>
+        <v>1.29</v>
       </c>
       <c r="H23" s="10" t="n">
-        <v>0.97</v>
+        <v>0.89</v>
       </c>
       <c r="I23" s="10" t="n">
-        <v>1.15</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6034,25 +6034,25 @@
         <v>73</v>
       </c>
       <c r="C24" s="10" t="n">
-        <v>1.29</v>
+        <v>1.31</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="F24" s="10" t="n">
         <v>0.11</v>
       </c>
       <c r="G24" s="10" t="n">
-        <v>0.47</v>
+        <v>0.48</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>0.68</v>
+        <v>0.54</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>0.79</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6112,7 +6112,7 @@
         <v>8</v>
       </c>
       <c r="H28" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I28" s="8" t="n">
         <v>3</v>
@@ -6141,7 +6141,7 @@
         <v>1</v>
       </c>
       <c r="H29" s="8" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I29" s="8" t="n">
         <v>2</v>
@@ -6170,7 +6170,7 @@
         <v>25</v>
       </c>
       <c r="H30" s="8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I30" s="8" t="n">
         <v>11</v>
@@ -6199,7 +6199,7 @@
         <v>2</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I31" s="8" t="n">
         <v>7</v>
@@ -6228,7 +6228,7 @@
         <v>10</v>
       </c>
       <c r="H32" s="8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I32" s="8" t="n">
         <v>8</v>
@@ -6257,7 +6257,7 @@
         <v>5</v>
       </c>
       <c r="H33" s="8" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I33" s="8" t="n">
         <v>3</v>
@@ -6286,7 +6286,7 @@
         <v>26</v>
       </c>
       <c r="H34" s="8" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I34" s="8" t="n">
         <v>14</v>
@@ -6315,7 +6315,7 @@
         <v>6</v>
       </c>
       <c r="H35" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I35" s="8" t="n">
         <v>14</v>
@@ -6460,7 +6460,7 @@
         <v>93</v>
       </c>
       <c r="H40" s="8" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="I40" s="8" t="n">
         <v>92</v>
@@ -6489,7 +6489,7 @@
         <v>18</v>
       </c>
       <c r="H41" s="8" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="I41" s="8" t="n">
         <v>20</v>
@@ -6518,7 +6518,7 @@
         <v>87</v>
       </c>
       <c r="H42" s="8" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I42" s="8" t="n">
         <v>79</v>
@@ -6547,7 +6547,7 @@
         <v>23</v>
       </c>
       <c r="H43" s="8" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="I43" s="8" t="n">
         <v>35</v>

</xml_diff>